<commit_message>
improved max size to reduce time
</commit_message>
<xml_diff>
--- a/case_studies/backbone/carriers_list.xlsx
+++ b/case_studies/backbone/carriers_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\case_studies\backbone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5993C8C3-FDA8-42C9-B91A-0703067DF7E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCCE35E1-1604-4AC1-99A3-CB007A028ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28020" yWindow="540" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-360" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="carriers" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>electricity</t>
   </si>
@@ -34,9 +34,6 @@
   </si>
   <si>
     <t>methane</t>
-  </si>
-  <si>
-    <t>heat</t>
   </si>
   <si>
     <t>CO2</t>
@@ -420,12 +417,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -470,12 +467,12 @@
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
@@ -520,22 +517,17 @@
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>